<commit_message>
equipamento para instalação do sensor
</commit_message>
<xml_diff>
--- a/Atividade 28-08-2025   Cronograma Modelo (GanttChart_modelo).xlsx
+++ b/Atividade 28-08-2025   Cronograma Modelo (GanttChart_modelo).xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antonio_j_jesus\Documents\vibracao_motor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F756E2F4-657F-498A-A0C6-C151B31CE05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEC959D-BD95-44FD-A718-518A18EB6771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GanttChart_pesquisa" sheetId="2" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="3" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="prevWBS" localSheetId="0">GanttChart_pesquisa!$A$1048573</definedName>
@@ -772,21 +773,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -817,6 +803,21 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1162,9 +1163,9 @@
       <c r="I1" s="2"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
@@ -1214,12 +1215,12 @@
       <c r="C4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="58">
         <v>45897</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
       <c r="I4" s="12" t="s">
         <v>2</v>
       </c>
@@ -1232,92 +1233,92 @@
       <c r="C5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="51">
+      <c r="D5" s="58">
         <v>45989</v>
       </c>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
       <c r="H5" s="12"/>
       <c r="I5" s="9"/>
       <c r="J5" s="14"/>
-      <c r="L5" s="46">
+      <c r="L5" s="60">
         <f>J4</f>
         <v>1</v>
       </c>
-      <c r="M5" s="47"/>
-      <c r="N5" s="46">
+      <c r="M5" s="57"/>
+      <c r="N5" s="60">
         <f>L5+1</f>
         <v>2</v>
       </c>
-      <c r="O5" s="47"/>
-      <c r="P5" s="46">
+      <c r="O5" s="57"/>
+      <c r="P5" s="60">
         <f>N5+1</f>
         <v>3</v>
       </c>
-      <c r="Q5" s="47"/>
-      <c r="R5" s="46">
+      <c r="Q5" s="57"/>
+      <c r="R5" s="60">
         <f>P5+1</f>
         <v>4</v>
       </c>
-      <c r="S5" s="47"/>
-      <c r="T5" s="46">
+      <c r="S5" s="57"/>
+      <c r="T5" s="60">
         <f>R5+1</f>
         <v>5</v>
       </c>
-      <c r="U5" s="47"/>
-      <c r="V5" s="46">
+      <c r="U5" s="57"/>
+      <c r="V5" s="60">
         <f>T5+1</f>
         <v>6</v>
       </c>
-      <c r="W5" s="47"/>
-      <c r="X5" s="46">
+      <c r="W5" s="57"/>
+      <c r="X5" s="60">
         <f>V5+1</f>
         <v>7</v>
       </c>
-      <c r="Y5" s="47"/>
-      <c r="Z5" s="46">
+      <c r="Y5" s="57"/>
+      <c r="Z5" s="60">
         <f>X5+1</f>
         <v>8</v>
       </c>
-      <c r="AA5" s="47"/>
-      <c r="AB5" s="46">
+      <c r="AA5" s="57"/>
+      <c r="AB5" s="60">
         <f>Z5+1</f>
         <v>9</v>
       </c>
-      <c r="AC5" s="47"/>
-      <c r="AD5" s="46">
+      <c r="AC5" s="57"/>
+      <c r="AD5" s="60">
         <f>AB5+1</f>
         <v>10</v>
       </c>
-      <c r="AE5" s="47"/>
-      <c r="AF5" s="46">
+      <c r="AE5" s="57"/>
+      <c r="AF5" s="60">
         <f>AD5+1</f>
         <v>11</v>
       </c>
-      <c r="AG5" s="47"/>
-      <c r="AH5" s="46">
+      <c r="AG5" s="57"/>
+      <c r="AH5" s="60">
         <f>AF5+1</f>
         <v>12</v>
       </c>
-      <c r="AI5" s="47"/>
-      <c r="AJ5" s="46">
+      <c r="AI5" s="57"/>
+      <c r="AJ5" s="60">
         <f>AH5+1</f>
         <v>13</v>
       </c>
-      <c r="AK5" s="47"/>
+      <c r="AK5" s="57"/>
     </row>
     <row r="6" spans="1:37" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="C6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
@@ -1618,10 +1619,10 @@
       <c r="AK8" s="27"/>
     </row>
     <row r="9" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="52" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="39"/>
@@ -1672,10 +1673,10 @@
       <c r="AK9" s="30"/>
     </row>
     <row r="10" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="46" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="39"/>
@@ -1726,7 +1727,7 @@
       <c r="AK10" s="30"/>
     </row>
     <row r="11" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="47" t="s">
         <v>26</v>
       </c>
       <c r="B11" s="29" t="s">
@@ -1782,10 +1783,10 @@
       <c r="AK11" s="30"/>
     </row>
     <row r="12" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="48" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="39"/>
@@ -1888,10 +1889,10 @@
       <c r="AK13" s="27"/>
     </row>
     <row r="14" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="48" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="39"/>
@@ -1942,10 +1943,10 @@
       <c r="AK14" s="30"/>
     </row>
     <row r="15" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
+      <c r="A15" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="55" t="s">
+      <c r="B15" s="48" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="39"/>
@@ -1996,25 +1997,25 @@
       <c r="AK15" s="30"/>
     </row>
     <row r="16" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="54" t="s">
+      <c r="A16" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="55" t="s">
+      <c r="B16" s="48" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="57">
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="50">
         <v>4</v>
       </c>
-      <c r="H16" s="57"/>
-      <c r="I16" s="56"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="49"/>
       <c r="J16" s="33"/>
-      <c r="K16" s="58"/>
+      <c r="K16" s="51"/>
       <c r="L16" s="44"/>
       <c r="M16" s="44"/>
       <c r="N16" s="44"/>
@@ -2043,10 +2044,10 @@
       <c r="AK16" s="30"/>
     </row>
     <row r="17" spans="1:37" ht="12.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="52" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="39"/>
@@ -2152,7 +2153,7 @@
       <c r="A19" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="62" t="s">
+      <c r="B19" s="55" t="s">
         <v>39</v>
       </c>
       <c r="C19" s="39"/>
@@ -2206,22 +2207,22 @@
       <c r="A20" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="52" t="s">
         <v>40</v>
       </c>
       <c r="C20" s="39"/>
       <c r="D20" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="E20" s="53"/>
+      <c r="F20" s="53"/>
       <c r="G20" s="32">
         <v>6</v>
       </c>
       <c r="H20" s="32"/>
-      <c r="I20" s="60"/>
+      <c r="I20" s="53"/>
       <c r="J20" s="33"/>
-      <c r="K20" s="61"/>
+      <c r="K20" s="54"/>
       <c r="L20" s="28"/>
       <c r="M20" s="28"/>
       <c r="N20" s="28"/>
@@ -2253,7 +2254,7 @@
       <c r="A21" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="52" t="s">
         <v>41</v>
       </c>
       <c r="C21" s="39"/>
@@ -2307,7 +2308,7 @@
       <c r="A22" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="59" t="s">
+      <c r="B22" s="52" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="39"/>
@@ -5582,11 +5583,6 @@
     <row r="997" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="N5:O5"/>
     <mergeCell ref="P5:Q5"/>
     <mergeCell ref="R5:S5"/>
     <mergeCell ref="D6:G6"/>
@@ -5599,6 +5595,11 @@
     <mergeCell ref="AB5:AC5"/>
     <mergeCell ref="AD5:AE5"/>
     <mergeCell ref="AF5:AG5"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="N5:O5"/>
   </mergeCells>
   <conditionalFormatting sqref="L7:AJ81">
     <cfRule type="expression" dxfId="4" priority="1">
@@ -5633,4 +5634,13 @@
   <drawing r:id="rId5"/>
   <legacyDrawing r:id="rId6"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA4A03AB-8290-46B4-8DFB-A74A3A038887}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>